<commit_message>
Prepare two-field account pilot and correct asymmetric reversion detection
</commit_message>
<xml_diff>
--- a/DQ_ENGINE/config/DQ_RDS_account_fields.xlsx
+++ b/DQ_ENGINE/config/DQ_RDS_account_fields.xlsx
@@ -405,9 +405,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A20"/>
   <cols>
-    <col min="1" max="1" width="120.83203125" customWidth="1"/>
+    <col min="1" max="1" width="135.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -432,7 +432,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>For each selected numeric field, agree all four movement/return settings before running.</v>
+        <v>Only PCKG_BALANCE_AMT and PCKG_REPAY_AMT are active for the pilot; the other 22 fields are retained as inactive.</v>
       </c>
     </row>
     <row r="6">
@@ -447,7 +447,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Blank numeric limits are intentional: no financial materiality assumptions were invented.</v>
+        <v>Pilot thresholds are provisional review limits, not approved financial materiality or automatic data-error rules.</v>
       </c>
     </row>
     <row r="9">
@@ -485,9 +485,34 @@
         <v>Account-level outputs remain in approved internal storage; do not upload customer results to GitHub.</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Pilot window in SAS file 06: 1 October 2025 to 31 March 2026 (six months).</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Balance: absolute jump 10000 and relative jump 0.50; return tolerance max(1000, 0.05 * original value magnitude).</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Repayment: absolute jump 250 and relative jump 0.50; return tolerance max(25, 0.05 * original value magnitude).</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Reversion: the first jump qualifies; the next movement reverses direction and returns within tolerance.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Remaining numeric fields need agreed units/limits; the two months-since counters need counter-specific checks before activation.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A20"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -533,7 +558,7 @@
         <v>IO_IND</v>
       </c>
       <c r="B2" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G2" t="str">
         <v>N</v>
@@ -544,7 +569,7 @@
         <v>IO_AT_ORIGINATION_IND</v>
       </c>
       <c r="B3" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G3" t="str">
         <v>Y</v>
@@ -555,7 +580,7 @@
         <v>REPAY_TYPE_CD</v>
       </c>
       <c r="B4" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G4" t="str">
         <v>N</v>
@@ -568,6 +593,18 @@
       <c r="B5" t="str">
         <v>Y</v>
       </c>
+      <c r="C5">
+        <v>10000</v>
+      </c>
+      <c r="D5">
+        <v>0.5</v>
+      </c>
+      <c r="E5">
+        <v>1000</v>
+      </c>
+      <c r="F5">
+        <v>0.05</v>
+      </c>
       <c r="G5" t="str">
         <v>N</v>
       </c>
@@ -577,7 +614,7 @@
         <v>PCKG_BOVO_VAL_AMT</v>
       </c>
       <c r="B6" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G6" t="str">
         <v>N</v>
@@ -588,7 +625,7 @@
         <v>MV_PCKG_LOAN_TO_INC_RT</v>
       </c>
       <c r="B7" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G7" t="str">
         <v>N</v>
@@ -599,7 +636,7 @@
         <v>CUTOVER_DT</v>
       </c>
       <c r="B8" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G8" t="str">
         <v>Y</v>
@@ -610,7 +647,7 @@
         <v>MV_PCKG_AVG_PAY_TO_BAL_L6M_RT</v>
       </c>
       <c r="B9" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G9" t="str">
         <v>N</v>
@@ -621,7 +658,7 @@
         <v>MV_PCKG_SAV_DEP_TO_REPAY_RT</v>
       </c>
       <c r="B10" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G10" t="str">
         <v>N</v>
@@ -632,7 +669,7 @@
         <v>MV_PCKG_SAV_DEP_TO_BALANCE_RT</v>
       </c>
       <c r="B11" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G11" t="str">
         <v>N</v>
@@ -643,7 +680,7 @@
         <v>MV_PROP_POSTCODE_NM</v>
       </c>
       <c r="B12" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G12" t="str">
         <v>N</v>
@@ -654,7 +691,7 @@
         <v>EVENT_DESCRIPTION</v>
       </c>
       <c r="B13" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G13" t="str">
         <v>N</v>
@@ -665,7 +702,7 @@
         <v>MTHS_SINCE_DETERIORATION_CNT</v>
       </c>
       <c r="B14" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G14" t="str">
         <v>N</v>
@@ -676,7 +713,7 @@
         <v>MV_PCKG_REPAY_TO_INC_RT</v>
       </c>
       <c r="B15" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G15" t="str">
         <v>N</v>
@@ -687,7 +724,7 @@
         <v>PCKG_FTB_CALC_IND</v>
       </c>
       <c r="B16" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G16" t="str">
         <v>N</v>
@@ -698,7 +735,7 @@
         <v>CHQ_LMT_UTIL_AVG_BAL_6M</v>
       </c>
       <c r="B17" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G17" t="str">
         <v>N</v>
@@ -709,7 +746,7 @@
         <v>MV_EXDAY_PAYREV</v>
       </c>
       <c r="B18" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G18" t="str">
         <v>N</v>
@@ -720,7 +757,7 @@
         <v>CUST_ALL_C_PYMTS_CR_AVG_L6M_AMT</v>
       </c>
       <c r="B19" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G19" t="str">
         <v>N</v>
@@ -731,7 +768,7 @@
         <v>PCKG_HI_INC_OCC_DESC</v>
       </c>
       <c r="B20" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G20" t="str">
         <v>N</v>
@@ -742,7 +779,7 @@
         <v>PCKG_2ND_INC_OCC_DESC</v>
       </c>
       <c r="B21" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G21" t="str">
         <v>N</v>
@@ -753,7 +790,7 @@
         <v>MV_CUST_ALL_MTHS_SNC_DIST_CNT</v>
       </c>
       <c r="B22" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G22" t="str">
         <v>N</v>
@@ -764,7 +801,7 @@
         <v>CUST_ALL_MT_MAX_DELINQ_BASE_RT</v>
       </c>
       <c r="B23" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G23" t="str">
         <v>N</v>
@@ -775,7 +812,7 @@
         <v>MV_PCKG_BAL_AMT_L6M_TO_L7T12M_RT</v>
       </c>
       <c r="B24" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="G24" t="str">
         <v>N</v>
@@ -787,6 +824,18 @@
       </c>
       <c r="B25" t="str">
         <v>Y</v>
+      </c>
+      <c r="C25">
+        <v>250</v>
+      </c>
+      <c r="D25">
+        <v>0.5</v>
+      </c>
+      <c r="E25">
+        <v>25</v>
+      </c>
+      <c r="F25">
+        <v>0.05</v>
       </c>
       <c r="G25" t="str">
         <v>N</v>
@@ -803,18 +852,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J25"/>
-  <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="38.83203125" customWidth="1"/>
-    <col min="4" max="4" width="40.83203125" customWidth="1"/>
-    <col min="5" max="5" width="42.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="90.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -970,7 +1007,7 @@
         <v>EXACT_NAME</v>
       </c>
       <c r="I5" t="str">
-        <v>TO_AGREE</v>
+        <v>PROVISIONAL_PILOT</v>
       </c>
       <c r="J5" t="str">
         <v>Uses CDAO package balance PCKG_BALANCE_AMT, not account BALANCE_AMT. Package membership/latest application/collateral changes may explain movements.</v>
@@ -1610,7 +1647,7 @@
         <v>EXACT_NAME</v>
       </c>
       <c r="I25" t="str">
-        <v>TO_AGREE</v>
+        <v>PROVISIONAL_PILOT</v>
       </c>
       <c r="J25" t="str">
         <v>Included following analyst confirmation. Package membership/repayment changes may explain movements.</v>
@@ -1627,12 +1664,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D3"/>
-  <cols>
-    <col min="1" max="1" width="26.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="95.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Select categorical and date account checks for full RDS history
</commit_message>
<xml_diff>
--- a/DQ_ENGINE/config/DQ_RDS_account_fields.xlsx
+++ b/DQ_ENGINE/config/DQ_RDS_account_fields.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A23"/>
   <cols>
     <col min="1" max="1" width="135.83203125" customWidth="1"/>
   </cols>
@@ -432,7 +432,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Only PCKG_BALANCE_AMT and PCKG_REPAY_AMT are active for the pilot; the other 22 fields are retained as inactive.</v>
+        <v>Current stage: all nine categorical fields and CUTOVER_DT are active; all 14 numeric fields are inactive.</v>
       </c>
     </row>
     <row r="6">
@@ -487,32 +487,47 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Pilot window in SAS file 06: 1 October 2025 to 31 March 2026 (six months).</v>
+        <v>Paused numeric balance limits retained: 10000 absolute / 0.50 relative jump; return max(1000, 0.05 * original magnitude).</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Balance: absolute jump 10000 and relative jump 0.50; return tolerance max(1000, 0.05 * original value magnitude).</v>
+        <v>Paused numeric repayment limits retained: 250 absolute / 0.50 relative jump; return max(25, 0.05 * original magnitude).</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Repayment: absolute jump 250 and relative jump 0.50; return tolerance max(25, 0.05 * original value magnitude).</v>
+        <v>Reversion: the first jump qualifies; the next movement reverses direction and returns within tolerance.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Reversion: the first jump qualifies; the next movement reverses direction and returns within tolerance.</v>
+        <v>Remaining numeric fields need agreed units/limits; the two months-since counters need counter-specific checks before activation.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Remaining numeric fields need agreed units/limits; the two months-since counters need counter-specific checks before activation.</v>
+        <v>Active categorical/date fields require no numeric movement limits.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>File 06 default date window: 1 January 2005 through 31 March 2026. Adjust to the agreed source scope if needed.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Detail export is capped at 10000 flagged rows per field; monthly summaries include all eligible observations.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Category reversions and temporary missing/special values are review flags; valid-to-valid fixed-field changes are enabled for IO_AT_ORIGINATION_IND and CUTOVER_DT.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A23"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -520,15 +535,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G25"/>
-  <cols>
-    <col min="1" max="1" width="42.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -558,7 +564,7 @@
         <v>IO_IND</v>
       </c>
       <c r="B2" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="G2" t="str">
         <v>N</v>
@@ -569,7 +575,7 @@
         <v>IO_AT_ORIGINATION_IND</v>
       </c>
       <c r="B3" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="G3" t="str">
         <v>Y</v>
@@ -580,7 +586,7 @@
         <v>REPAY_TYPE_CD</v>
       </c>
       <c r="B4" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="G4" t="str">
         <v>N</v>
@@ -591,7 +597,7 @@
         <v>PCKG_BALANCE_AMT</v>
       </c>
       <c r="B5" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="C5">
         <v>10000</v>
@@ -636,7 +642,7 @@
         <v>CUTOVER_DT</v>
       </c>
       <c r="B8" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="G8" t="str">
         <v>Y</v>
@@ -680,7 +686,7 @@
         <v>MV_PROP_POSTCODE_NM</v>
       </c>
       <c r="B12" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="G12" t="str">
         <v>N</v>
@@ -691,7 +697,7 @@
         <v>EVENT_DESCRIPTION</v>
       </c>
       <c r="B13" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="G13" t="str">
         <v>N</v>
@@ -724,7 +730,7 @@
         <v>PCKG_FTB_CALC_IND</v>
       </c>
       <c r="B16" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="G16" t="str">
         <v>N</v>
@@ -746,7 +752,7 @@
         <v>MV_EXDAY_PAYREV</v>
       </c>
       <c r="B18" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="G18" t="str">
         <v>N</v>
@@ -768,7 +774,7 @@
         <v>PCKG_HI_INC_OCC_DESC</v>
       </c>
       <c r="B20" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="G20" t="str">
         <v>N</v>
@@ -779,7 +785,7 @@
         <v>PCKG_2ND_INC_OCC_DESC</v>
       </c>
       <c r="B21" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="G21" t="str">
         <v>N</v>
@@ -823,7 +829,7 @@
         <v>PCKG_REPAY_AMT</v>
       </c>
       <c r="B25" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="C25">
         <v>250</v>

</xml_diff>

<commit_message>
Persist account-level DQ results and add Teradata review views
</commit_message>
<xml_diff>
--- a/DQ_ENGINE/config/DQ_RDS_account_fields.xlsx
+++ b/DQ_ENGINE/config/DQ_RDS_account_fields.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A25"/>
   <cols>
     <col min="1" max="1" width="135.83203125" customWidth="1"/>
   </cols>
@@ -517,7 +517,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Detail export is capped at 10000 flagged rows per field; monthly summaries include all eligible observations.</v>
+        <v>SAS detail export is capped at 10000 rows per field; Teradata saves all flagged detail and uncapped monthly summaries.</v>
       </c>
     </row>
     <row r="23">
@@ -525,9 +525,19 @@
         <v>Category reversions and temporary missing/special values are review flags; valid-to-valid fixed-field changes are enabled for IO_AT_ORIGINATION_IND and CUTOVER_DT.</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>One-time persistence deployment: run setup/22_create_account_results.sql and results/96_dq_account_review.sql before current SAS 07.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Run numbers and progress are saved in Teradata; review DQ_ACCOUNT_REVIEW and DQ_ACCOUNT_DETAIL_REVIEW after SAS closes.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A25"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>